<commit_message>
updated code with vectorized functions where possible
</commit_message>
<xml_diff>
--- a/Two Stage Deterministic equivalent/MVP_random_normal_forecast_data.xlsx
+++ b/Two Stage Deterministic equivalent/MVP_random_normal_forecast_data.xlsx
@@ -1,88 +1,80 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27425"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Two Stage Deterministic equivalent/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{B517B12B-BA54-4E69-90F1-E7D24CA29F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{745A137A-E6AA-4D0B-B87C-CF0B5034E8D4}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_48F5423BA231921FD2FE31D2F8F2D3C274DF5CAF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F56EF5D1-CEB3-4646-AC4D-1425FDCA1D97}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A5115543-AC87-4E62-8A65-1522949D5C3B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Medium_Demand" sheetId="11" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
-    <t>PCV</t>
+    <t>Measles</t>
+  </si>
+  <si>
+    <t>Mumps</t>
+  </si>
+  <si>
+    <t>Rubella</t>
+  </si>
+  <si>
+    <t>Diphtheria</t>
+  </si>
+  <si>
+    <t>Tetanus</t>
+  </si>
+  <si>
+    <t>Pertussis</t>
+  </si>
+  <si>
+    <t>Hepatitis_B</t>
+  </si>
+  <si>
+    <t>Hib</t>
+  </si>
+  <si>
+    <t>Polio</t>
+  </si>
+  <si>
+    <t>HPV</t>
   </si>
   <si>
     <t>Rotavirus</t>
   </si>
   <si>
-    <t>HPV</t>
-  </si>
-  <si>
-    <t>Polio</t>
-  </si>
-  <si>
-    <t>Hib</t>
-  </si>
-  <si>
-    <t>Hepatitis_B</t>
-  </si>
-  <si>
-    <t>Pertussis</t>
-  </si>
-  <si>
-    <t>Tetanus</t>
-  </si>
-  <si>
-    <t>Diphtheria</t>
-  </si>
-  <si>
-    <t>Rubella</t>
-  </si>
-  <si>
-    <t>Mumps</t>
-  </si>
-  <si>
-    <t>Measles</t>
+    <t>PCV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -95,12 +87,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -109,13 +116,15 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -182,7 +191,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$2</c:f>
+              <c:f>Sheet1!$A$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -205,7 +214,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -244,39 +253,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$2:$K$2</c:f>
+              <c:f>Sheet1!$B$2:$K$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>2193753000.4354081</c:v>
+                <c:pt idx="0">
+                  <c:v>456988291.83199197</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2482447605.6538076</c:v>
+                  <c:v>504766004.65349662</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2224864354.7325668</c:v>
+                  <c:v>400132317.81236303</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3001900115.2997451</c:v>
+                  <c:v>557389329.98345613</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3856232647.2174392</c:v>
+                  <c:v>819661666.94559038</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2630553742.5824852</c:v>
+                  <c:v>606924894.08955026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4643119414.0215321</c:v>
+                  <c:v>824890632.70418549</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4222254596.7234898</c:v>
+                  <c:v>744187065.23033166</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4633165906.4723825</c:v>
+                  <c:v>842958744.62559807</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5498863006.7956276</c:v>
+                  <c:v>1039520613.031508</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -284,7 +293,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000000-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -293,7 +302,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$3</c:f>
+              <c:f>Sheet1!$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -316,7 +325,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -355,39 +364,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$3:$K$3</c:f>
+              <c:f>Sheet1!$B$3:$K$3</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>148033771.45748568</c:v>
+                <c:pt idx="0">
+                  <c:v>27610410.454955179</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>161206713.06136197</c:v>
+                  <c:v>31456115.845126491</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>117208412.41314472</c:v>
+                  <c:v>25440504.82264585</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>148640175.98283696</c:v>
+                  <c:v>34891385.835228801</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>176522706.02080849</c:v>
+                  <c:v>34199574.56645909</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>192110701.16516086</c:v>
+                  <c:v>45425225.086442113</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>215905454.40391913</c:v>
+                  <c:v>50572225.946408428</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>227456460.89563364</c:v>
+                  <c:v>52454214.398228332</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>174284987.16961703</c:v>
+                  <c:v>51743076.905033208</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>291918686.07048541</c:v>
+                  <c:v>66412251.58737497</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -395,7 +404,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000001-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -404,7 +413,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$4</c:f>
+              <c:f>Sheet1!$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -427,7 +436,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -466,39 +475,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$4:$K$4</c:f>
+              <c:f>Sheet1!$B$4:$K$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>2068022529.0354507</c:v>
+                <c:pt idx="0">
+                  <c:v>334662138.65108901</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2232390400.0215197</c:v>
+                  <c:v>435805281.36144561</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2252478090.9749894</c:v>
+                  <c:v>425469603.27958709</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1530899599.4567842</c:v>
+                  <c:v>392456130.84345448</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2414012318.5134659</c:v>
+                  <c:v>521679550.85319543</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3235841602.290309</c:v>
+                  <c:v>595613650.48656154</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2753831163.1930885</c:v>
+                  <c:v>568782370.10033309</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3346778361.0728683</c:v>
+                  <c:v>703391002.2361927</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3255824639.7373919</c:v>
+                  <c:v>673773442.88245189</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4613103288.4044304</c:v>
+                  <c:v>901857281.32807469</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -506,7 +515,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000002-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -515,7 +524,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$5</c:f>
+              <c:f>Sheet1!$A$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -538,7 +547,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -577,39 +586,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$5:$K$5</c:f>
+              <c:f>Sheet1!$B$5:$K$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>3225677141.2824931</c:v>
+                <c:pt idx="0">
+                  <c:v>618629991.68856335</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3472604543.6621571</c:v>
+                  <c:v>759051596.65785444</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4412122494.3728189</c:v>
+                  <c:v>891719281.4203999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4146548785.6124916</c:v>
+                  <c:v>780326497.94468141</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5044636632.4064884</c:v>
+                  <c:v>868544983.26769829</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6879524787.3561077</c:v>
+                  <c:v>1274086579.30251</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6475114404.8840313</c:v>
+                  <c:v>1307956207.70295</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7743738600.5743971</c:v>
+                  <c:v>1456789607.6260481</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>7823347470.4904556</c:v>
+                  <c:v>1486857112.8824561</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9425228547.4780102</c:v>
+                  <c:v>1859254080.628412</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -617,7 +626,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000003-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -626,7 +635,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$6</c:f>
+              <c:f>Sheet1!$A$6</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -649,7 +658,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -688,39 +697,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$6:$K$6</c:f>
+              <c:f>Sheet1!$B$6:$K$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>3311948869.4447746</c:v>
+                <c:pt idx="0">
+                  <c:v>636907993.10709012</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3254314848.7791567</c:v>
+                  <c:v>661078181.17900443</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3059283514.5879788</c:v>
+                  <c:v>620874156.66733134</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3294893995.5552497</c:v>
+                  <c:v>679267208.88045061</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3139586088.5604753</c:v>
+                  <c:v>683702116.40520537</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3234826415.3742423</c:v>
+                  <c:v>649930806.54251289</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3386775719.43503</c:v>
+                  <c:v>657181174.98658299</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3449613314.6039228</c:v>
+                  <c:v>690802365.22840953</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3705341024.4236155</c:v>
+                  <c:v>723089566.01546466</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4077768323.7741251</c:v>
+                  <c:v>773696551.80895531</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -728,7 +737,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000004-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -737,7 +746,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$7</c:f>
+              <c:f>Sheet1!$A$7</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -760,7 +769,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -799,39 +808,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$7:$K$7</c:f>
+              <c:f>Sheet1!$B$7:$K$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>1791213415.1436608</c:v>
+                <c:pt idx="0">
+                  <c:v>355905487.99301869</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1788588073.0324996</c:v>
+                  <c:v>346971868.0685212</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2001768159.8621287</c:v>
+                  <c:v>379759761.11259258</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1656991889.7593882</c:v>
+                  <c:v>346876344.26808709</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1758155587.6133962</c:v>
+                  <c:v>370698693.90286028</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2058046460.0058386</c:v>
+                  <c:v>390326544.50291282</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1950655225.3114288</c:v>
+                  <c:v>379811000.56437278</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1761637267.4890099</c:v>
+                  <c:v>378893141.26294172</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2085664829.1307664</c:v>
+                  <c:v>420509152.81217641</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2092209705.5477076</c:v>
+                  <c:v>407415991.66574228</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -839,7 +848,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000005-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -848,7 +857,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$8</c:f>
+              <c:f>Sheet1!$A$8</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -873,7 +882,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -912,39 +921,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$8:$K$8</c:f>
+              <c:f>Sheet1!$B$8:$K$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>2149662743.9159384</c:v>
+                <c:pt idx="0">
+                  <c:v>416786632.40658623</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1835775642.6935086</c:v>
+                  <c:v>376336078.24478221</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2173549455.6622858</c:v>
+                  <c:v>427306336.3340373</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2126178394.8287535</c:v>
+                  <c:v>451295491.94730818</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1686784437.350596</c:v>
+                  <c:v>335802465.04568309</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2361862855.9895239</c:v>
+                  <c:v>464982691.69720173</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1876434508.5756853</c:v>
+                  <c:v>425166587.75108051</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1876535318.347899</c:v>
+                  <c:v>375123367.29025352</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1873460866.4937403</c:v>
+                  <c:v>341179423.08773232</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2018980053.6389189</c:v>
+                  <c:v>390746346.00944769</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -952,7 +961,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000006-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -961,7 +970,7 @@
           <c:order val="7"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$9</c:f>
+              <c:f>Sheet1!$A$9</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -986,7 +995,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1025,39 +1034,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$9:$K$9</c:f>
+              <c:f>Sheet1!$B$9:$K$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>1626979034.7221804</c:v>
+                <c:pt idx="0">
+                  <c:v>318969070.69684142</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1468100191.1072607</c:v>
+                  <c:v>310949924.45530641</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1546309220.9837394</c:v>
+                  <c:v>320149875.32736701</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1578132152.8123863</c:v>
+                  <c:v>329003035.86656392</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1902417782.1091771</c:v>
+                  <c:v>363473504.96695769</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1818997913.4738753</c:v>
+                  <c:v>364550583.272291</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1796167410.3389797</c:v>
+                  <c:v>362914318.94792348</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1922223295.9816129</c:v>
+                  <c:v>387291721.38924408</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2110749530.6028271</c:v>
+                  <c:v>415460021.39644021</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2043268844.1202445</c:v>
+                  <c:v>431887868.8753525</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1065,7 +1074,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000007-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000007-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1074,7 +1083,7 @@
           <c:order val="8"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$10</c:f>
+              <c:f>Sheet1!$A$10</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1099,7 +1108,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1138,39 +1147,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$10:$K$10</c:f>
+              <c:f>Sheet1!$B$10:$K$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>2981440820.5268941</c:v>
+                <c:pt idx="0">
+                  <c:v>595880933.40664709</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3222503077.1441646</c:v>
+                  <c:v>674604017.69397986</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3183968758.8969879</c:v>
+                  <c:v>692411485.13128829</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3927589732.6214876</c:v>
+                  <c:v>742881436.42496645</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3610271136.1670451</c:v>
+                  <c:v>735593541.14244485</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4085941739.7177744</c:v>
+                  <c:v>780055824.23650444</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3949882145.8642845</c:v>
+                  <c:v>827341791.21000338</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4415701022.3859406</c:v>
+                  <c:v>870604378.79102552</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4632657247.3324785</c:v>
+                  <c:v>910332454.75333846</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4686743013.1313334</c:v>
+                  <c:v>971102781.75564933</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1178,7 +1187,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000008-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1187,7 +1196,7 @@
           <c:order val="9"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$11</c:f>
+              <c:f>Sheet1!$A$11</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1212,7 +1221,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1251,39 +1260,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$11:$K$11</c:f>
+              <c:f>Sheet1!$B$11:$K$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>133927318.76325457</c:v>
+                <c:pt idx="0">
+                  <c:v>27690723.562539682</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>190892852.44147769</c:v>
+                  <c:v>36553091.879725322</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>203725677.24655816</c:v>
+                  <c:v>39789603.464589372</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>205254515.5219686</c:v>
+                  <c:v>43546281.525075123</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>289993431.62897962</c:v>
+                  <c:v>56652918.306098439</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>296311868.30840051</c:v>
+                  <c:v>58955585.60182704</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>324463850.00519639</c:v>
+                  <c:v>67704760.675126404</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>379141066.07647508</c:v>
+                  <c:v>75502244.190795645</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>416064711.62045133</c:v>
+                  <c:v>80059981.322654754</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>437678253.87556583</c:v>
+                  <c:v>89737383.843908623</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1291,7 +1300,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{00000009-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1300,7 +1309,7 @@
           <c:order val="10"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$12</c:f>
+              <c:f>Sheet1!$A$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1325,7 +1334,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1364,39 +1373,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$12:$K$12</c:f>
+              <c:f>Sheet1!$B$12:$K$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>1185675164.1658239</c:v>
+                <c:pt idx="0">
+                  <c:v>227320847.73904499</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1129154410.7562034</c:v>
+                  <c:v>236696375.40990961</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1025625297.7154663</c:v>
+                  <c:v>256269619.83443049</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1959229609.5782306</c:v>
+                  <c:v>345222902.38778228</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1655915737.5303214</c:v>
+                  <c:v>349931540.09940833</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1146940529.2793186</c:v>
+                  <c:v>313469855.04360598</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2177767784.3901701</c:v>
+                  <c:v>515835076.2928465</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2776763352.0710831</c:v>
+                  <c:v>550584828.84340847</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3237468749.2225704</c:v>
+                  <c:v>686348335.41897893</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3505086165.8343639</c:v>
+                  <c:v>714486721.91353762</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1404,7 +1413,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000A-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{0000000A-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1413,7 +1422,7 @@
           <c:order val="11"/>
           <c:tx>
             <c:strRef>
-              <c:f>Medium_Demand!$A$13</c:f>
+              <c:f>Sheet1!$A$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1438,7 +1447,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Medium_Demand!$B$1:$K$1</c:f>
+              <c:f>Sheet1!$B$1:$K$1</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1477,39 +1486,39 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Medium_Demand!$B$13:$K$13</c:f>
+              <c:f>Sheet1!$B$13:$K$13</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0" formatCode="0.00E+00">
-                  <c:v>1168392719.0900152</c:v>
+                <c:pt idx="0">
+                  <c:v>234044249.86782131</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1289760304.9576085</c:v>
+                  <c:v>262482765.92490149</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1326994356.9669383</c:v>
+                  <c:v>257785690.8972761</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1560669221.6935143</c:v>
+                  <c:v>300005578.16007048</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1920571658.7645125</c:v>
+                  <c:v>353147975.20503223</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1815841145.9009511</c:v>
+                  <c:v>332550505.78506631</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2432423626.5146174</c:v>
+                  <c:v>449500912.66469669</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1834023748.8449767</c:v>
+                  <c:v>374756851.15936881</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2522514570.7589173</c:v>
+                  <c:v>490248480.75143731</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2657543162.4369335</c:v>
+                  <c:v>478920704.48757309</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1517,7 +1526,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-116E-4A7C-BFB8-BD566A996D42}"/>
+              <c16:uniqueId val="{0000000B-64DC-4C8D-A405-02DC1B30059F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1530,11 +1539,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="1756156240"/>
-        <c:axId val="1756163440"/>
+        <c:axId val="1758403104"/>
+        <c:axId val="291274464"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="1756156240"/>
+        <c:axId val="1758403104"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1577,7 +1586,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1756163440"/>
+        <c:crossAx val="291274464"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1585,7 +1594,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1756163440"/>
+        <c:axId val="291274464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1605,7 +1614,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1636,7 +1645,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1756156240"/>
+        <c:crossAx val="1758403104"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2284,22 +2293,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>66674</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>14286</xdr:rowOff>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>228599</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>152399</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>100012</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{752021FE-A6B0-A7B6-0A0E-5D06F0A6BF4B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{341E3A82-DD6E-876E-CF3B-BF7525AB209F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2320,14 +2329,10 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2335,44 +2340,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -2400,31 +2405,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -2452,26 +2440,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2480,623 +2451,624 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF7ED23-11A8-43C7-BCD0-EFF91A7F3943}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B1">
+      <c r="B1" s="1">
         <v>1</v>
       </c>
-      <c r="C1">
+      <c r="C1" s="1">
         <v>2</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="1">
         <v>3</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="1">
         <v>4</v>
       </c>
-      <c r="F1">
+      <c r="F1" s="1">
         <v>5</v>
       </c>
-      <c r="G1">
+      <c r="G1" s="1">
         <v>6</v>
       </c>
-      <c r="H1">
+      <c r="H1" s="1">
         <v>7</v>
       </c>
-      <c r="I1">
+      <c r="I1" s="1">
         <v>8</v>
       </c>
-      <c r="J1">
+      <c r="J1" s="1">
         <v>9</v>
       </c>
-      <c r="K1">
+      <c r="K1" s="1">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="1">
-        <v>2193753000.4354081</v>
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>456988291.83199197</v>
       </c>
       <c r="C2">
-        <v>2482447605.6538076</v>
+        <v>504766004.65349662</v>
       </c>
       <c r="D2">
-        <v>2224864354.7325668</v>
+        <v>400132317.81236303</v>
       </c>
       <c r="E2">
-        <v>3001900115.2997451</v>
+        <v>557389329.98345613</v>
       </c>
       <c r="F2">
-        <v>3856232647.2174392</v>
+        <v>819661666.94559038</v>
       </c>
       <c r="G2">
-        <v>2630553742.5824852</v>
+        <v>606924894.08955026</v>
       </c>
       <c r="H2">
-        <v>4643119414.0215321</v>
+        <v>824890632.70418549</v>
       </c>
       <c r="I2">
-        <v>4222254596.7234898</v>
+        <v>744187065.23033166</v>
       </c>
       <c r="J2">
-        <v>4633165906.4723825</v>
+        <v>842958744.62559807</v>
       </c>
       <c r="K2">
-        <v>5498863006.7956276</v>
+        <v>1039520613.031508</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="1">
-        <v>148033771.45748568</v>
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>27610410.454955179</v>
       </c>
       <c r="C3">
-        <v>161206713.06136197</v>
+        <v>31456115.845126491</v>
       </c>
       <c r="D3">
-        <v>117208412.41314472</v>
+        <v>25440504.82264585</v>
       </c>
       <c r="E3">
-        <v>148640175.98283696</v>
+        <v>34891385.835228801</v>
       </c>
       <c r="F3">
-        <v>176522706.02080849</v>
+        <v>34199574.56645909</v>
       </c>
       <c r="G3">
-        <v>192110701.16516086</v>
+        <v>45425225.086442113</v>
       </c>
       <c r="H3">
-        <v>215905454.40391913</v>
+        <v>50572225.946408428</v>
       </c>
       <c r="I3">
-        <v>227456460.89563364</v>
+        <v>52454214.398228332</v>
       </c>
       <c r="J3">
-        <v>174284987.16961703</v>
+        <v>51743076.905033208</v>
       </c>
       <c r="K3">
-        <v>291918686.07048541</v>
+        <v>66412251.58737497</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="1">
-        <v>2068022529.0354507</v>
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>334662138.65108901</v>
       </c>
       <c r="C4">
-        <v>2232390400.0215197</v>
+        <v>435805281.36144561</v>
       </c>
       <c r="D4">
-        <v>2252478090.9749894</v>
+        <v>425469603.27958709</v>
       </c>
       <c r="E4">
-        <v>1530899599.4567842</v>
+        <v>392456130.84345448</v>
       </c>
       <c r="F4">
-        <v>2414012318.5134659</v>
+        <v>521679550.85319543</v>
       </c>
       <c r="G4">
-        <v>3235841602.290309</v>
+        <v>595613650.48656154</v>
       </c>
       <c r="H4">
-        <v>2753831163.1930885</v>
+        <v>568782370.10033309</v>
       </c>
       <c r="I4">
-        <v>3346778361.0728683</v>
+        <v>703391002.2361927</v>
       </c>
       <c r="J4">
-        <v>3255824639.7373919</v>
+        <v>673773442.88245189</v>
       </c>
       <c r="K4">
-        <v>4613103288.4044304</v>
+        <v>901857281.32807469</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1">
-        <v>3225677141.2824931</v>
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>618629991.68856335</v>
       </c>
       <c r="C5">
-        <v>3472604543.6621571</v>
+        <v>759051596.65785444</v>
       </c>
       <c r="D5">
-        <v>4412122494.3728189</v>
+        <v>891719281.4203999</v>
       </c>
       <c r="E5">
-        <v>4146548785.6124916</v>
+        <v>780326497.94468141</v>
       </c>
       <c r="F5">
-        <v>5044636632.4064884</v>
+        <v>868544983.26769829</v>
       </c>
       <c r="G5">
-        <v>6879524787.3561077</v>
+        <v>1274086579.30251</v>
       </c>
       <c r="H5">
-        <v>6475114404.8840313</v>
+        <v>1307956207.70295</v>
       </c>
       <c r="I5">
-        <v>7743738600.5743971</v>
+        <v>1456789607.6260481</v>
       </c>
       <c r="J5">
-        <v>7823347470.4904556</v>
+        <v>1486857112.8824561</v>
       </c>
       <c r="K5">
-        <v>9425228547.4780102</v>
+        <v>1859254080.628412</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="1">
-        <v>3311948869.4447746</v>
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>636907993.10709012</v>
       </c>
       <c r="C6">
-        <v>3254314848.7791567</v>
+        <v>661078181.17900443</v>
       </c>
       <c r="D6">
-        <v>3059283514.5879788</v>
+        <v>620874156.66733134</v>
       </c>
       <c r="E6">
-        <v>3294893995.5552497</v>
+        <v>679267208.88045061</v>
       </c>
       <c r="F6">
-        <v>3139586088.5604753</v>
+        <v>683702116.40520537</v>
       </c>
       <c r="G6">
-        <v>3234826415.3742423</v>
+        <v>649930806.54251289</v>
       </c>
       <c r="H6">
-        <v>3386775719.43503</v>
+        <v>657181174.98658299</v>
       </c>
       <c r="I6">
-        <v>3449613314.6039228</v>
+        <v>690802365.22840953</v>
       </c>
       <c r="J6">
-        <v>3705341024.4236155</v>
+        <v>723089566.01546466</v>
       </c>
       <c r="K6">
-        <v>4077768323.7741251</v>
+        <v>773696551.80895531</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1">
-        <v>1791213415.1436608</v>
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>355905487.99301869</v>
       </c>
       <c r="C7">
-        <v>1788588073.0324996</v>
+        <v>346971868.0685212</v>
       </c>
       <c r="D7">
-        <v>2001768159.8621287</v>
+        <v>379759761.11259258</v>
       </c>
       <c r="E7">
-        <v>1656991889.7593882</v>
+        <v>346876344.26808709</v>
       </c>
       <c r="F7">
-        <v>1758155587.6133962</v>
+        <v>370698693.90286028</v>
       </c>
       <c r="G7">
-        <v>2058046460.0058386</v>
+        <v>390326544.50291282</v>
       </c>
       <c r="H7">
-        <v>1950655225.3114288</v>
+        <v>379811000.56437278</v>
       </c>
       <c r="I7">
-        <v>1761637267.4890099</v>
+        <v>378893141.26294172</v>
       </c>
       <c r="J7">
-        <v>2085664829.1307664</v>
+        <v>420509152.81217641</v>
       </c>
       <c r="K7">
-        <v>2092209705.5477076</v>
+        <v>407415991.66574228</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1">
-        <v>2149662743.9159384</v>
+      <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>416786632.40658623</v>
       </c>
       <c r="C8">
-        <v>1835775642.6935086</v>
+        <v>376336078.24478221</v>
       </c>
       <c r="D8">
-        <v>2173549455.6622858</v>
+        <v>427306336.3340373</v>
       </c>
       <c r="E8">
-        <v>2126178394.8287535</v>
+        <v>451295491.94730818</v>
       </c>
       <c r="F8">
-        <v>1686784437.350596</v>
+        <v>335802465.04568309</v>
       </c>
       <c r="G8">
-        <v>2361862855.9895239</v>
+        <v>464982691.69720173</v>
       </c>
       <c r="H8">
-        <v>1876434508.5756853</v>
+        <v>425166587.75108051</v>
       </c>
       <c r="I8">
-        <v>1876535318.347899</v>
+        <v>375123367.29025352</v>
       </c>
       <c r="J8">
-        <v>1873460866.4937403</v>
+        <v>341179423.08773232</v>
       </c>
       <c r="K8">
-        <v>2018980053.6389189</v>
+        <v>390746346.00944769</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="1">
-        <v>1626979034.7221804</v>
+      <c r="A9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>318969070.69684142</v>
       </c>
       <c r="C9">
-        <v>1468100191.1072607</v>
+        <v>310949924.45530641</v>
       </c>
       <c r="D9">
-        <v>1546309220.9837394</v>
+        <v>320149875.32736701</v>
       </c>
       <c r="E9">
-        <v>1578132152.8123863</v>
+        <v>329003035.86656392</v>
       </c>
       <c r="F9">
-        <v>1902417782.1091771</v>
+        <v>363473504.96695769</v>
       </c>
       <c r="G9">
-        <v>1818997913.4738753</v>
+        <v>364550583.272291</v>
       </c>
       <c r="H9">
-        <v>1796167410.3389797</v>
+        <v>362914318.94792348</v>
       </c>
       <c r="I9">
-        <v>1922223295.9816129</v>
+        <v>387291721.38924408</v>
       </c>
       <c r="J9">
-        <v>2110749530.6028271</v>
+        <v>415460021.39644021</v>
       </c>
       <c r="K9">
-        <v>2043268844.1202445</v>
+        <v>431887868.8753525</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1">
-        <v>2981440820.5268941</v>
+      <c r="A10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>595880933.40664709</v>
       </c>
       <c r="C10">
-        <v>3222503077.1441646</v>
+        <v>674604017.69397986</v>
       </c>
       <c r="D10">
-        <v>3183968758.8969879</v>
+        <v>692411485.13128829</v>
       </c>
       <c r="E10">
-        <v>3927589732.6214876</v>
+        <v>742881436.42496645</v>
       </c>
       <c r="F10">
-        <v>3610271136.1670451</v>
+        <v>735593541.14244485</v>
       </c>
       <c r="G10">
-        <v>4085941739.7177744</v>
+        <v>780055824.23650444</v>
       </c>
       <c r="H10">
-        <v>3949882145.8642845</v>
+        <v>827341791.21000338</v>
       </c>
       <c r="I10">
-        <v>4415701022.3859406</v>
+        <v>870604378.79102552</v>
       </c>
       <c r="J10">
-        <v>4632657247.3324785</v>
+        <v>910332454.75333846</v>
       </c>
       <c r="K10">
-        <v>4686743013.1313334</v>
+        <v>971102781.75564933</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B11" s="1">
-        <v>133927318.76325457</v>
+      <c r="A11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>27690723.562539682</v>
       </c>
       <c r="C11">
-        <v>190892852.44147769</v>
+        <v>36553091.879725322</v>
       </c>
       <c r="D11">
-        <v>203725677.24655816</v>
+        <v>39789603.464589372</v>
       </c>
       <c r="E11">
-        <v>205254515.5219686</v>
+        <v>43546281.525075123</v>
       </c>
       <c r="F11">
-        <v>289993431.62897962</v>
+        <v>56652918.306098439</v>
       </c>
       <c r="G11">
-        <v>296311868.30840051</v>
+        <v>58955585.60182704</v>
       </c>
       <c r="H11">
-        <v>324463850.00519639</v>
+        <v>67704760.675126404</v>
       </c>
       <c r="I11">
-        <v>379141066.07647508</v>
+        <v>75502244.190795645</v>
       </c>
       <c r="J11">
-        <v>416064711.62045133</v>
+        <v>80059981.322654754</v>
       </c>
       <c r="K11">
-        <v>437678253.87556583</v>
+        <v>89737383.843908623</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" s="1">
-        <v>1185675164.1658239</v>
+      <c r="A12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>227320847.73904499</v>
       </c>
       <c r="C12">
-        <v>1129154410.7562034</v>
+        <v>236696375.40990961</v>
       </c>
       <c r="D12">
-        <v>1025625297.7154663</v>
+        <v>256269619.83443049</v>
       </c>
       <c r="E12">
-        <v>1959229609.5782306</v>
+        <v>345222902.38778228</v>
       </c>
       <c r="F12">
-        <v>1655915737.5303214</v>
+        <v>349931540.09940833</v>
       </c>
       <c r="G12">
-        <v>1146940529.2793186</v>
+        <v>313469855.04360598</v>
       </c>
       <c r="H12">
-        <v>2177767784.3901701</v>
+        <v>515835076.2928465</v>
       </c>
       <c r="I12">
-        <v>2776763352.0710831</v>
+        <v>550584828.84340847</v>
       </c>
       <c r="J12">
-        <v>3237468749.2225704</v>
+        <v>686348335.41897893</v>
       </c>
       <c r="K12">
-        <v>3505086165.8343639</v>
+        <v>714486721.91353762</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B13" s="1">
-        <v>1168392719.0900152</v>
+      <c r="A13" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>234044249.86782131</v>
       </c>
       <c r="C13">
-        <v>1289760304.9576085</v>
+        <v>262482765.92490149</v>
       </c>
       <c r="D13">
-        <v>1326994356.9669383</v>
+        <v>257785690.8972761</v>
       </c>
       <c r="E13">
-        <v>1560669221.6935143</v>
+        <v>300005578.16007048</v>
       </c>
       <c r="F13">
-        <v>1920571658.7645125</v>
+        <v>353147975.20503223</v>
       </c>
       <c r="G13">
-        <v>1815841145.9009511</v>
+        <v>332550505.78506631</v>
       </c>
       <c r="H13">
-        <v>2432423626.5146174</v>
+        <v>449500912.66469669</v>
       </c>
       <c r="I13">
-        <v>1834023748.8449767</v>
+        <v>374756851.15936881</v>
       </c>
       <c r="J13">
-        <v>2522514570.7589173</v>
+        <v>490248480.75143731</v>
       </c>
       <c r="K13">
-        <v>2657543162.4369335</v>
+        <v>478920704.48757309</v>
       </c>
     </row>
   </sheetData>

</xml_diff>